<commit_message>
Add SI percentile distribution data and per-city box plot
- Per-city stats now include P10/P25/P50/P75/P90, IQR, std
- shade_index_data.xlsx: expanded Shade Index sheet + new
  'SI Percentiles' sheet for easy custom plotting in Excel
- New plot 05_si_distribution_per_city.png: per-city box plot
  (P25-P75 box, P10-P90 whiskers), reveals shade homogeneity
- Report updated with distribution shape section and full percentile table

Key insight: most cities show right-skewed SI distributions with mean
> median, indicating that "high SI" cities like KFS (mean 0.274,
median 0.154) owe much of their averaged shade to ~10-25% of
heavily shaded pixels.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shade_index_data.xlsx
+++ b/shade_index_data.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shade Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI Percentiles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,45 +436,75 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>std_SI</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>min_SI</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>P10_SI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>P25_SI</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>median_SI</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>min_SI</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>P75_SI</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>P90_SI</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>max_SI</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>IQR_SI</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>max_exposure</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>mean_exposure</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>median_exposure</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>min_exposure</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>n_pixels</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>street_area_m2</t>
         </is>
@@ -494,30 +525,48 @@
         <v>0.2741791753715095</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1537577849284646</v>
+        <v>0.2937744880099078</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
+        <v>0.01224213822833362</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.04070351441720887</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.1537577849284646</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.4372752526799895</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.8483071740746936</v>
+      </c>
+      <c r="K2" t="n">
         <v>0.9317805145347923</v>
       </c>
-      <c r="G2" t="n">
+      <c r="L2" t="n">
+        <v>0.3965717382627806</v>
+      </c>
+      <c r="M2" t="n">
         <v>4606.834411621094</v>
       </c>
-      <c r="H2" t="n">
+      <c r="N2" t="n">
         <v>3343.736351569728</v>
       </c>
-      <c r="I2" t="n">
+      <c r="O2" t="n">
         <v>3898.497756958008</v>
       </c>
-      <c r="J2" t="n">
+      <c r="P2" t="n">
         <v>314.2758731842041</v>
       </c>
-      <c r="K2" t="n">
+      <c r="Q2" t="n">
         <v>9767015</v>
       </c>
-      <c r="L2" t="n">
+      <c r="R2" t="n">
         <v>2441753.75</v>
       </c>
     </row>
@@ -536,30 +585,48 @@
         <v>0.2519532104256198</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1436741358325506</v>
+        <v>0.2577214726685976</v>
       </c>
       <c r="E3" t="n">
         <v>9.325209975097337e-06</v>
       </c>
       <c r="F3" t="n">
+        <v>0.02162735468178312</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.05261362420466439</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1436741358325506</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.3854524231567156</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.74876337136015</v>
+      </c>
+      <c r="K3" t="n">
         <v>0.9338216948708887</v>
       </c>
-      <c r="G3" t="n">
+      <c r="L3" t="n">
+        <v>0.3328387989520512</v>
+      </c>
+      <c r="M3" t="n">
         <v>5065.967529296875</v>
       </c>
-      <c r="H3" t="n">
+      <c r="N3" t="n">
         <v>3789.580746378582</v>
       </c>
-      <c r="I3" t="n">
+      <c r="O3" t="n">
         <v>4338.119022369385</v>
       </c>
-      <c r="J3" t="n">
+      <c r="P3" t="n">
         <v>335.2571449279785</v>
       </c>
-      <c r="K3" t="n">
+      <c r="Q3" t="n">
         <v>42732450</v>
       </c>
-      <c r="L3" t="n">
+      <c r="R3" t="n">
         <v>10683112.5</v>
       </c>
     </row>
@@ -578,30 +645,48 @@
         <v>0.2297827683502874</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1007639189539434</v>
+        <v>0.2715085811000756</v>
       </c>
       <c r="E4" t="n">
         <v>-1.037821397975591e-05</v>
       </c>
       <c r="F4" t="n">
+        <v>0.01299814882882801</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.03825751646290332</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1007639189539434</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.3152273998877505</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.7738733458584074</v>
+      </c>
+      <c r="K4" t="n">
         <v>0.9342922510540309</v>
       </c>
-      <c r="G4" t="n">
+      <c r="L4" t="n">
+        <v>0.2769698834248472</v>
+      </c>
+      <c r="M4" t="n">
         <v>5064.349128723145</v>
       </c>
-      <c r="H4" t="n">
+      <c r="N4" t="n">
         <v>3900.648966032775</v>
       </c>
-      <c r="I4" t="n">
+      <c r="O4" t="n">
         <v>4554.045463562012</v>
       </c>
-      <c r="J4" t="n">
+      <c r="P4" t="n">
         <v>332.7669811248779</v>
       </c>
-      <c r="K4" t="n">
+      <c r="Q4" t="n">
         <v>11950193</v>
       </c>
-      <c r="L4" t="n">
+      <c r="R4" t="n">
         <v>2987548.25</v>
       </c>
     </row>
@@ -620,30 +705,48 @@
         <v>0.2273591375652459</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1066468407874093</v>
+        <v>0.2587163832949868</v>
       </c>
       <c r="E5" t="n">
         <v>4.534718404114457e-07</v>
       </c>
       <c r="F5" t="n">
+        <v>0.01290396305417574</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.03608411513648824</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.1066468407874093</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.331310564940085</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.7350938622756636</v>
+      </c>
+      <c r="K5" t="n">
         <v>0.9199844858545387</v>
       </c>
-      <c r="G5" t="n">
+      <c r="L5" t="n">
+        <v>0.2952264498035968</v>
+      </c>
+      <c r="M5" t="n">
         <v>5064.146324157715</v>
       </c>
-      <c r="H5" t="n">
+      <c r="N5" t="n">
         <v>3912.766383393007</v>
       </c>
-      <c r="I5" t="n">
+      <c r="O5" t="n">
         <v>4524.071117401123</v>
       </c>
-      <c r="J5" t="n">
+      <c r="P5" t="n">
         <v>405.2102718353271</v>
       </c>
-      <c r="K5" t="n">
+      <c r="Q5" t="n">
         <v>8336044</v>
       </c>
-      <c r="L5" t="n">
+      <c r="R5" t="n">
         <v>2084011</v>
       </c>
     </row>
@@ -662,30 +765,48 @@
         <v>0.2096918360781797</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08291999809228967</v>
+        <v>0.2632637436276495</v>
       </c>
       <c r="E6" t="n">
         <v>1.038364471561692e-05</v>
       </c>
       <c r="F6" t="n">
+        <v>0.01168090976936618</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.03156988777378489</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.08291999809228967</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.2783826707348822</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.7351749748829682</v>
+      </c>
+      <c r="K6" t="n">
         <v>0.9342268821399232</v>
       </c>
-      <c r="G6" t="n">
+      <c r="L6" t="n">
+        <v>0.2468127829610973</v>
+      </c>
+      <c r="M6" t="n">
         <v>5064.639434814453</v>
       </c>
-      <c r="H6" t="n">
+      <c r="N6" t="n">
         <v>4002.625892654256</v>
       </c>
-      <c r="I6" t="n">
+      <c r="O6" t="n">
         <v>4644.679542541504</v>
       </c>
-      <c r="J6" t="n">
+      <c r="P6" t="n">
         <v>333.1171264648438</v>
       </c>
-      <c r="K6" t="n">
+      <c r="Q6" t="n">
         <v>7654857</v>
       </c>
-      <c r="L6" t="n">
+      <c r="R6" t="n">
         <v>1913714.25</v>
       </c>
     </row>
@@ -704,30 +825,48 @@
         <v>0.1932597759760895</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0853285955283718</v>
+        <v>0.2408633784460567</v>
       </c>
       <c r="E7" t="n">
         <v>4.368267661436498e-05</v>
       </c>
       <c r="F7" t="n">
+        <v>0.01317208692778848</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.03149314190411556</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0853285955283718</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.2580526114259561</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.6092918889464453</v>
+      </c>
+      <c r="K7" t="n">
         <v>0.9343073184817454</v>
       </c>
-      <c r="G7" t="n">
+      <c r="L7" t="n">
+        <v>0.2265594695218406</v>
+      </c>
+      <c r="M7" t="n">
         <v>5065.516738891602</v>
       </c>
-      <c r="H7" t="n">
+      <c r="N7" t="n">
         <v>4086.556108730279</v>
       </c>
-      <c r="I7" t="n">
+      <c r="O7" t="n">
         <v>4633.283309936523</v>
       </c>
-      <c r="J7" t="n">
+      <c r="P7" t="n">
         <v>332.7673778533936</v>
       </c>
-      <c r="K7" t="n">
+      <c r="Q7" t="n">
         <v>18177185</v>
       </c>
-      <c r="L7" t="n">
+      <c r="R7" t="n">
         <v>4544296.25</v>
       </c>
     </row>
@@ -746,30 +885,48 @@
         <v>0.1835536057097672</v>
       </c>
       <c r="D8" t="n">
-        <v>0.09694179678263792</v>
+        <v>0.2177066658937197</v>
       </c>
       <c r="E8" t="n">
         <v>1.10696423758494e-05</v>
       </c>
       <c r="F8" t="n">
+        <v>0.01524523767187025</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.04007508664464787</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.09694179678263792</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.2361068688483212</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.4832214862249437</v>
+      </c>
+      <c r="K8" t="n">
         <v>0.9301732037472699</v>
       </c>
-      <c r="G8" t="n">
+      <c r="L8" t="n">
+        <v>0.1960317822036733</v>
+      </c>
+      <c r="M8" t="n">
         <v>5066.44002532959</v>
       </c>
-      <c r="H8" t="n">
+      <c r="N8" t="n">
         <v>4136.47669056806</v>
       </c>
-      <c r="I8" t="n">
+      <c r="O8" t="n">
         <v>4575.290225982666</v>
       </c>
-      <c r="J8" t="n">
+      <c r="P8" t="n">
         <v>353.7732753753662</v>
       </c>
-      <c r="K8" t="n">
+      <c r="Q8" t="n">
         <v>6293530</v>
       </c>
-      <c r="L8" t="n">
+      <c r="R8" t="n">
         <v>1573382.5</v>
       </c>
     </row>
@@ -788,30 +945,48 @@
         <v>0.1755611279240797</v>
       </c>
       <c r="D9" t="n">
-        <v>0.08014285288817991</v>
+        <v>0.2204037726018331</v>
       </c>
       <c r="E9" t="n">
         <v>2.913823564210105e-06</v>
       </c>
       <c r="F9" t="n">
+        <v>0.01191384361912198</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.03196017513046379</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.08014285288817991</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.217238692797732</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.542011788688648</v>
+      </c>
+      <c r="K9" t="n">
         <v>0.9242981349701085</v>
       </c>
-      <c r="G9" t="n">
+      <c r="L9" t="n">
+        <v>0.1852785176672682</v>
+      </c>
+      <c r="M9" t="n">
         <v>5066.497024536133</v>
       </c>
-      <c r="H9" t="n">
+      <c r="N9" t="n">
         <v>4177.017092284575</v>
       </c>
-      <c r="I9" t="n">
+      <c r="O9" t="n">
         <v>4660.453498840332</v>
       </c>
-      <c r="J9" t="n">
+      <c r="P9" t="n">
         <v>383.5432739257812</v>
       </c>
-      <c r="K9" t="n">
+      <c r="Q9" t="n">
         <v>13071733</v>
       </c>
-      <c r="L9" t="n">
+      <c r="R9" t="n">
         <v>3267933.25</v>
       </c>
     </row>
@@ -830,30 +1005,48 @@
         <v>0.1708976530742735</v>
       </c>
       <c r="D10" t="n">
-        <v>0.06187929258882097</v>
+        <v>0.2379354884261044</v>
       </c>
       <c r="E10" t="n">
         <v>-3.267103976245522e-07</v>
       </c>
       <c r="F10" t="n">
+        <v>0.005208161211279982</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.02221119560410767</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.06187929258882097</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.1953883342870316</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.5782101597846004</v>
+      </c>
+      <c r="K10" t="n">
         <v>0.9334432217482627</v>
       </c>
-      <c r="G10" t="n">
+      <c r="L10" t="n">
+        <v>0.1731771386829239</v>
+      </c>
+      <c r="M10" t="n">
         <v>5067.419418334961</v>
       </c>
-      <c r="H10" t="n">
+      <c r="N10" t="n">
         <v>4201.409332598516</v>
       </c>
-      <c r="I10" t="n">
+      <c r="O10" t="n">
         <v>4753.851089477539</v>
       </c>
-      <c r="J10" t="n">
+      <c r="P10" t="n">
         <v>337.271110534668</v>
       </c>
-      <c r="K10" t="n">
+      <c r="Q10" t="n">
         <v>6149053</v>
       </c>
-      <c r="L10" t="n">
+      <c r="R10" t="n">
         <v>1537263.25</v>
       </c>
     </row>
@@ -872,30 +1065,48 @@
         <v>0.1365451127614682</v>
       </c>
       <c r="D11" t="n">
-        <v>0.04793998331471921</v>
+        <v>0.204949906982576</v>
       </c>
       <c r="E11" t="n">
         <v>-4.005278721974648e-05</v>
       </c>
       <c r="F11" t="n">
+        <v>0.003918601410256795</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.01370764184741913</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.04793998331471921</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1532457380177824</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.4179101558704119</v>
+      </c>
+      <c r="K11" t="n">
         <v>0.9340723647972838</v>
       </c>
-      <c r="G11" t="n">
+      <c r="L11" t="n">
+        <v>0.1395380961703633</v>
+      </c>
+      <c r="M11" t="n">
         <v>5062.860572814941</v>
       </c>
-      <c r="H11" t="n">
+      <c r="N11" t="n">
         <v>4371.551705004334</v>
       </c>
-      <c r="I11" t="n">
+      <c r="O11" t="n">
         <v>4820.147121429443</v>
       </c>
-      <c r="J11" t="n">
+      <c r="P11" t="n">
         <v>333.7824249267578</v>
       </c>
-      <c r="K11" t="n">
+      <c r="Q11" t="n">
         <v>21310342</v>
       </c>
-      <c r="L11" t="n">
+      <c r="R11" t="n">
         <v>5327391.22477172</v>
       </c>
     </row>
@@ -914,30 +1125,48 @@
         <v>0.1214810430809439</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02198006602006863</v>
+        <v>0.231312705699933</v>
       </c>
       <c r="E12" t="n">
         <v>2.211758402093089e-06</v>
       </c>
       <c r="F12" t="n">
+        <v>0.007314238297838505</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.01233231707080351</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.02198006602006863</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.06618187978046153</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.4514222575206334</v>
+      </c>
+      <c r="K12" t="n">
         <v>0.9324672201762686</v>
       </c>
-      <c r="G12" t="n">
+      <c r="L12" t="n">
+        <v>0.05384956270965802</v>
+      </c>
+      <c r="M12" t="n">
         <v>5060.372673034668</v>
       </c>
-      <c r="H12" t="n">
+      <c r="N12" t="n">
         <v>4445.633322336113</v>
       </c>
-      <c r="I12" t="n">
+      <c r="O12" t="n">
         <v>4949.145347595215</v>
       </c>
-      <c r="J12" t="n">
+      <c r="P12" t="n">
         <v>341.7410335540771</v>
       </c>
-      <c r="K12" t="n">
+      <c r="Q12" t="n">
         <v>6853617</v>
       </c>
-      <c r="L12" t="n">
+      <c r="R12" t="n">
         <v>1713404.25</v>
       </c>
     </row>
@@ -956,30 +1185,48 @@
         <v>0.1009425810995412</v>
       </c>
       <c r="D13" t="n">
-        <v>0.03438269227189739</v>
+        <v>0.1659910647460085</v>
       </c>
       <c r="E13" t="n">
         <v>6.545156880854996e-05</v>
       </c>
       <c r="F13" t="n">
+        <v>0.007774633322138791</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.01594134082474208</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.03438269227189739</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.09881357692410109</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.2742837161856295</v>
+      </c>
+      <c r="K13" t="n">
         <v>0.933988345211847</v>
       </c>
-      <c r="G13" t="n">
+      <c r="L13" t="n">
+        <v>0.08287223609935901</v>
+      </c>
+      <c r="M13" t="n">
         <v>5056.378051757812</v>
       </c>
-      <c r="H13" t="n">
+      <c r="N13" t="n">
         <v>4545.97420019831</v>
       </c>
-      <c r="I13" t="n">
+      <c r="O13" t="n">
         <v>4882.526161193848</v>
       </c>
-      <c r="J13" t="n">
+      <c r="P13" t="n">
         <v>333.7798824310303</v>
       </c>
-      <c r="K13" t="n">
+      <c r="Q13" t="n">
         <v>31698477</v>
       </c>
-      <c r="L13" t="n">
+      <c r="R13" t="n">
         <v>7924619.25</v>
       </c>
     </row>
@@ -998,30 +1245,48 @@
         <v>0.09522718477239102</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03094703803884735</v>
+        <v>0.1802896977484067</v>
       </c>
       <c r="E14" t="n">
         <v>4.017890122987033e-05</v>
       </c>
       <c r="F14" t="n">
+        <v>0.008372096097073678</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.01654760719189752</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.03094703803884735</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.06745015965447987</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.2574903195361118</v>
+      </c>
+      <c r="K14" t="n">
         <v>0.9305342008067753</v>
       </c>
-      <c r="G14" t="n">
+      <c r="L14" t="n">
+        <v>0.05090255246258235</v>
+      </c>
+      <c r="M14" t="n">
         <v>5070.325134277344</v>
       </c>
-      <c r="H14" t="n">
+      <c r="N14" t="n">
         <v>4587.492345859417</v>
       </c>
-      <c r="I14" t="n">
+      <c r="O14" t="n">
         <v>4913.413589477539</v>
       </c>
-      <c r="J14" t="n">
+      <c r="P14" t="n">
         <v>352.2141876220703</v>
       </c>
-      <c r="K14" t="n">
+      <c r="Q14" t="n">
         <v>2718725</v>
       </c>
-      <c r="L14" t="n">
+      <c r="R14" t="n">
         <v>679681.25</v>
       </c>
     </row>
@@ -1040,30 +1305,48 @@
         <v>0.08295121901132006</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0238808690211505</v>
+        <v>0.1609772426620437</v>
       </c>
       <c r="E15" t="n">
         <v>1.899848994568742e-05</v>
       </c>
       <c r="F15" t="n">
+        <v>0.004112870217645059</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.01074137953206833</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.0238808690211505</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.07085594452964583</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.1973153043026138</v>
+      </c>
+      <c r="K15" t="n">
         <v>0.9284498363516513</v>
       </c>
-      <c r="G15" t="n">
+      <c r="L15" t="n">
+        <v>0.0601145649975775</v>
+      </c>
+      <c r="M15" t="n">
         <v>4685.623733520508</v>
       </c>
-      <c r="H15" t="n">
+      <c r="N15" t="n">
         <v>4296.945532996609</v>
       </c>
-      <c r="I15" t="n">
+      <c r="O15" t="n">
         <v>4573.72696685791</v>
       </c>
-      <c r="J15" t="n">
+      <c r="P15" t="n">
         <v>335.2571449279785</v>
       </c>
-      <c r="K15" t="n">
+      <c r="Q15" t="n">
         <v>8152715</v>
       </c>
-      <c r="L15" t="n">
+      <c r="R15" t="n">
         <v>2038178.75</v>
       </c>
     </row>
@@ -1082,30 +1365,48 @@
         <v>0.07540363018810263</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02659613418008255</v>
+        <v>0.1366614473364721</v>
       </c>
       <c r="E16" t="n">
         <v>8.53570372161272e-08</v>
       </c>
       <c r="F16" t="n">
+        <v>0.004409161186316846</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.01150435746252532</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.02659613418008255</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.06633740970739796</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.1745475179653838</v>
+      </c>
+      <c r="K16" t="n">
         <v>0.9282186476155909</v>
       </c>
-      <c r="G16" t="n">
+      <c r="L16" t="n">
+        <v>0.05483305224487264</v>
+      </c>
+      <c r="M16" t="n">
         <v>5094.781898498535</v>
       </c>
-      <c r="H16" t="n">
+      <c r="N16" t="n">
         <v>4710.616848335113</v>
       </c>
-      <c r="I16" t="n">
+      <c r="O16" t="n">
         <v>4959.280395507812</v>
       </c>
-      <c r="J16" t="n">
+      <c r="P16" t="n">
         <v>365.710334777832</v>
       </c>
-      <c r="K16" t="n">
+      <c r="Q16" t="n">
         <v>9906380</v>
       </c>
-      <c r="L16" t="n">
+      <c r="R16" t="n">
         <v>2476595</v>
       </c>
     </row>
@@ -1124,30 +1425,48 @@
         <v>0.07067767191232406</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01788167307707589</v>
+        <v>0.1645803780881361</v>
       </c>
       <c r="E17" t="n">
         <v>1.880119911534806e-06</v>
       </c>
       <c r="F17" t="n">
+        <v>0.003245443438020579</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.007123966869032272</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.01788167307707589</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.04615652794531794</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.1472933248518969</v>
+      </c>
+      <c r="K17" t="n">
         <v>0.9287099715457989</v>
       </c>
-      <c r="G17" t="n">
+      <c r="L17" t="n">
+        <v>0.03903256107628567</v>
+      </c>
+      <c r="M17" t="n">
         <v>5072.41219329834</v>
       </c>
-      <c r="H17" t="n">
+      <c r="N17" t="n">
         <v>4713.905908496327</v>
       </c>
-      <c r="I17" t="n">
+      <c r="O17" t="n">
         <v>4981.708976745605</v>
       </c>
-      <c r="J17" t="n">
+      <c r="P17" t="n">
         <v>361.6124095916748</v>
       </c>
-      <c r="K17" t="n">
+      <c r="Q17" t="n">
         <v>6373119</v>
       </c>
-      <c r="L17" t="n">
+      <c r="R17" t="n">
         <v>1593279.75</v>
       </c>
     </row>
@@ -1166,30 +1485,48 @@
         <v>0.06662326426514956</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01702109427290011</v>
+        <v>0.1581562857233948</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
+        <v>0.003067972799277729</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.007291390771645645</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.01702109427290011</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.0435236454267105</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.1437448779727136</v>
+      </c>
+      <c r="K18" t="n">
         <v>0.9344437820279423</v>
       </c>
-      <c r="G18" t="n">
+      <c r="L18" t="n">
+        <v>0.03623225465506485</v>
+      </c>
+      <c r="M18" t="n">
         <v>5076.128868103027</v>
       </c>
-      <c r="H18" t="n">
+      <c r="N18" t="n">
         <v>4737.940593079445</v>
       </c>
-      <c r="I18" t="n">
+      <c r="O18" t="n">
         <v>4989.727600097656</v>
       </c>
-      <c r="J18" t="n">
+      <c r="P18" t="n">
         <v>332.7718105316162</v>
       </c>
-      <c r="K18" t="n">
+      <c r="Q18" t="n">
         <v>34372573</v>
       </c>
-      <c r="L18" t="n">
+      <c r="R18" t="n">
         <v>8593143.25</v>
       </c>
     </row>
@@ -1208,30 +1545,48 @@
         <v>0.04092917218804359</v>
       </c>
       <c r="D19" t="n">
-        <v>0.01275926828384399</v>
+        <v>0.1040304526686668</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
+        <v>0.001229465007781982</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.004111945629119873</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.01275926828384399</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.02844569087028503</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.07798576354980469</v>
+      </c>
+      <c r="K19" t="n">
         <v>0.9289379715919495</v>
       </c>
-      <c r="G19" t="n">
+      <c r="L19" t="n">
+        <v>0.02433374524116516</v>
+      </c>
+      <c r="M19" t="n">
         <v>5073.70458984375</v>
       </c>
-      <c r="H19" t="n">
+      <c r="N19" t="n">
         <v>4866.04248046875</v>
       </c>
-      <c r="I19" t="n">
+      <c r="O19" t="n">
         <v>5008.9677734375</v>
       </c>
-      <c r="J19" t="n">
+      <c r="P19" t="n">
         <v>360.5477600097656</v>
       </c>
-      <c r="K19" t="n">
+      <c r="Q19" t="n">
         <v>6502266</v>
       </c>
-      <c r="L19" t="n">
+      <c r="R19" t="n">
         <v>1625566.5</v>
       </c>
     </row>
@@ -1246,6 +1601,543 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>city_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>P10_SI</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>P25_SI</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>median_SI</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>P75_SI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>P90_SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KFS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kfar Saba</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.01224213822833362</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.04070351441720887</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1537577849284646</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.4372752526799895</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.8483071740746936</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TLV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.02162735468178312</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.05261362420466439</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1436741358325506</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.3854524231567156</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.74876337136015</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HRZ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Herzliya</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.01299814882882801</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.03825751646290332</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.1007639189539434</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.3152273998877505</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.7738733458584074</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Raanana</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.01290396305417574</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.03608411513648824</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1066468407874093</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.331310564940085</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.7350938622756636</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HDS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hod HaSharon</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.01168090976936618</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.03156988777378489</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.08291999809228967</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2783826707348822</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.7351749748829682</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PTV</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Petah Tikva</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.01317208692778848</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.03149314190411556</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0853285955283718</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2580526114259561</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.6092918889464453</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BTY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bat Yam</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.01524523767187025</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.04007508664464787</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.09694179678263792</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2361068688483212</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.4832214862249437</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Holon</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.01191384361912198</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.03196017513046379</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.08014285288817991</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.217238692797732</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.542011788688648</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NSZ</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ness Ziona</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.005208161211279982</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.02221119560410767</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.06187929258882097</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1953883342870316</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.5782101597846004</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NTN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Netanya</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.003918601410256795</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.01370764184741913</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.04793998331471921</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1532457380177824</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.4179101558704119</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PHK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pardes Hanna-Karkur</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.007314238297838505</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.01233231707080351</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.02198006602006863</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.06618187978046153</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.4514222575206334</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HAI</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Haifa</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.007774633322138791</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.01594134082474208</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.03438269227189739</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.09881357692410109</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.2742837161856295</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BTR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Beitar Ilit</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.008372096097073678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.01654760719189752</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.03094703803884735</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.06745015965447987</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.2574903195361118</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AKO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Akko</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.004112870217645059</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.01074137953206833</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0238808690211505</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.07085594452964583</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1973153043026138</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ELT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Eilat</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.004409161186316846</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.01150435746252532</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.02659613418008255</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.06633740970739796</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.1745475179653838</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SDR</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sderot</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.003245443438020579</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.007123966869032272</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.01788167307707589</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.04615652794531794</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.1472933248518969</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BSV</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Beersheva</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.003067972799277729</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.007291390771645645</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.01702109427290011</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0435236454267105</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.1437448779727136</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NTV</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Netivot</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.001229465007781982</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.004111945629119873</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.01275926828384399</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.02844569087028503</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.07798576354980469</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Add per-street-segment SI distribution (segments >= 250 m^2)
For each city's street_segments file:
- Strip Z if 3D, reproject to EPSG:2039
- Filter segments with area < 250 m^2
- For each kept segment, mask raster and compute mean SI
- Aggregate to per-segment SI distribution: mean, std,
  P10/P25/P50/P75/P90, IQR

New 'SI Per Street Segment' sheet in shade_index_data.xlsx with
all 18 cities. Note: per-segment mean SI is generally higher than
per-pixel mean SI because averaging smooths individual dark/light
pixels into per-street values.

Top cities (per-segment mean SI):
  KFS 0.296 (1714/2144 segments kept)
  TLV 0.275 (7222/8441)
  HRZ 0.255 (2055/2242)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shade_index_data.xlsx
+++ b/shade_index_data.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shade Index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI Percentiles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI Per Street Segment" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2138,6 +2139,956 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>city_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>seg_n_kept</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>seg_n_total</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>seg_mean_SI</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>seg_std_SI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>seg_min_SI</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>seg_P10_SI</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>seg_P25_SI</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>seg_median_SI</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>seg_P75_SI</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>seg_P90_SI</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>seg_max_SI</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>seg_IQR_SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KFS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kfar Saba</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1714</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2144</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2964388431519126</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1640597150123438</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.00165276211696059</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.08000006254850626</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1710884360704817</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.2884225950381882</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.409262532113597</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.5139212197209345</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.7830025692030802</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.2381740960431153</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TLV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>7222</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8441</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.2749478868508611</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1513117745224496</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.00147278161894449</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.09936217786209126</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1644142926994133</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.2516341474135599</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3619821804364691</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.4777244291944494</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.8319613521286424</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1975678877370558</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HRZ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Herzliya</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2055</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2242</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2545853619846032</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1494737794170328</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.00108345976251952</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.07898049132601863</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1471605571062466</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.2325882101954144</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.3354627600549281</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.4596281759253951</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.8480990624015247</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.1883022029486815</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RAN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Raanana</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1267</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1389</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.2451917761655367</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1356929437494528</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.001271458049165967</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.06588282999985698</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.1418598836612229</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.2373107325617729</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.3326171050702973</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.425404163189055</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.7287487640634526</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1907572214090744</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HDS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hod HaSharon</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1416</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1588</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.2228460014591871</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1415932233902972</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0005490935498450065</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.06268337289566697</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.1183790575054268</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.2035076251768151</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.3004029450368649</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.4163662978893621</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.8632936378826332</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.1820238875314382</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PTV</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Petah Tikva</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2841</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3093</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.2113290751435565</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1373256581822054</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.001308706986358314</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.05141237468318681</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.104674495515712</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.1910429655995604</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.2894626370144889</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.3998678948829981</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.7891511992789784</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.1847881414987769</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BTY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bat Yam</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1059</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1121</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1948717357755156</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.1156573603970714</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.001941262117334878</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.06733111290428938</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.1122784869100203</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.1777154915745199</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.2554987896494271</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.3412230572689784</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.7486975729181169</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.1432203027394067</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HOL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Holon</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1836</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2439</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1854915068853855</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1119802476531221</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.002027907931756512</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.06308088502190276</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.1040802291326577</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.1660405623802421</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.2465751316942494</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.3293605781007446</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.7583997456876908</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.1424949025615917</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NSZ</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ness Ziona</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1178</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1414</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1856340301405033</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.121755714091647</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0002130210696198837</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.04374748964868878</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.09473847646619382</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.1638407674754479</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.2526735271761907</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.3473308888728263</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.7362722783368185</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.1579350507099969</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NTN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Netanya</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2895</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4023</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1520843435763943</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1173108974758486</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.000498034847434712</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.02084095632197734</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.05977519292690649</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.1285413281626704</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.222821805513623</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.3084146687014183</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.7249165983460036</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.1630466125867165</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PHK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pardes Hanna-Karkur</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1452</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1660</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1188996007509384</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.0981924724671617</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.001322885783589781</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.02228596158444905</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.04660109286034428</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.09119963418697875</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.1662654259721879</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.2534597726878509</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.6697438796471368</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.1196643331118436</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HAI</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Haifa</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6494</v>
+      </c>
+      <c r="D13" t="n">
+        <v>8489</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.1177600775142088</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.1102746202393871</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.002489425537603391</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.02104032946124962</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.04063168559004583</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.08266177744566761</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.1600065932036038</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.2579804368492194</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.8353523515197249</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.119374907613558</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BTR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Beitar Ilit</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>402</v>
+      </c>
+      <c r="D14" t="n">
+        <v>478</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.09029976958809691</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.07204523532984232</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.003822228465059565</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.01671134735780217</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.03448267060584106</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.06946690250153749</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.1238937436224154</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.1866302213036255</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.3781809621906229</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.08941107301657433</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AKO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Akko</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1121</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1814</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.09176926854315361</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.08025163044210769</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.001284667712246217</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.02130376094368545</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.03901461966607819</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.06868439256723813</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.115988667655662</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.1824896992655882</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.7244307014591295</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.07697404798958382</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ELT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Eilat</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1737</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2538</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0856706124086505</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.07227093573446504</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.00112727710695467</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.01543894846963833</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.03540699996820053</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.06805077520844108</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.1171508646763376</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.1688095484156457</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.6330424651108896</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.08174386470813709</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SDR</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sderot</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1262</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1467</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.07619955667941469</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.08644958623887862</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0006764986920642851</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.004145057361954437</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.01693215883550525</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.05128647753396272</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.1036150786530424</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.17564789403784</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.8053992954700351</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.08668291981753717</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BSV</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Beersheva</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5506</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7173</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.07057084231270935</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0698996057476489</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0004338646228851404</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.01037788338340872</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.02435751325501621</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.04906721065591619</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.09358894662099371</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.1535749849217079</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.7241806432778346</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.06923143336597751</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NTV</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Netivot</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1205</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1554</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.04825807531271033</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.058568275566197</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0003626989782787859</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.00317691289819777</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.01075051911175251</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.03168264776468277</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.0638161301612854</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.1097039684653282</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.7472904324531555</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.05306561104953289</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>